<commit_message>
relation works but from java, not tested from python
</commit_message>
<xml_diff>
--- a/uploads/z-FriedrichKarlStroher.xlsx
+++ b/uploads/z-FriedrichKarlStroher.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t xml:space="preserve">property</t>
   </si>
@@ -28,6 +28,12 @@
     <t xml:space="preserve">text</t>
   </si>
   <si>
+    <t xml:space="preserve">Objekt-ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Varianter Name        </t>
   </si>
   <si>
@@ -107,6 +113,12 @@
   </si>
   <si>
     <t xml:space="preserve">Person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RELATION_authorOf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Object1</t>
   </si>
 </sst>
 </file>
@@ -203,19 +215,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -409,18 +421,18 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="39.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="39.13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -428,7 +440,7 @@
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -444,36 +456,36 @@
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -481,7 +493,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -489,39 +501,39 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="1" t="n">
+      <c r="B12" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="2" t="n">
         <v>118852051</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -532,97 +544,109 @@
       <c r="A15" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
+      <c r="A16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
+      <c r="A17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1"/>
-      <c r="B27" s="4"/>
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
+      <c r="A28" s="2"/>
+      <c r="B28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1"/>
-      <c r="B30" s="1"/>
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="1"/>
-      <c r="B32" s="1"/>
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1"/>
+      <c r="A33" s="2"/>
+      <c r="B33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1"/>
-      <c r="B34" s="1"/>
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="2"/>
+      <c r="B36" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B7" r:id="rId1" display="Maler | Bildhauer | Grafiker"/>
-    <hyperlink ref="B8" r:id="rId2" display="Malerei. Zeichnung. Graphik | Plastik"/>
-    <hyperlink ref="B9" r:id="rId3" display="Ströher, Peter  | Ströher, Charlotte"/>
-    <hyperlink ref="B13" r:id="rId4" display="Wikimedia Commons |  Deutsche Nationalbibliothek (DNB) |  Wikipedia-Personenartikel"/>
-    <hyperlink ref="B14" r:id="rId5" display="Literatur von Karl Friedrich Ströher in der RPB | Literatur über Karl Friedrich Ströher in der RPB"/>
+    <hyperlink ref="B8" r:id="rId1" display="Maler | Bildhauer | Grafiker"/>
+    <hyperlink ref="B9" r:id="rId2" display="Malerei. Zeichnung. Graphik | Plastik"/>
+    <hyperlink ref="B10" r:id="rId3" display="Ströher, Peter  | Ströher, Charlotte"/>
+    <hyperlink ref="B14" r:id="rId4" display="Wikimedia Commons |  Deutsche Nationalbibliothek (DNB) |  Wikipedia-Personenartikel"/>
+    <hyperlink ref="B15" r:id="rId5" display="Literatur von Karl Friedrich Ströher in der RPB | Literatur über Karl Friedrich Ströher in der RPB"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>